<commit_message>
📊 Actualizar COMISIONES_ASESORES_DASHBOARD.xlsx — 30-03-2026, 5:00:53 p. m.
</commit_message>
<xml_diff>
--- a/datos/COMISIONES_ASESORES_DASHBOARD.xlsx
+++ b/datos/COMISIONES_ASESORES_DASHBOARD.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/df502c28020c5b60/Documentos/GIM/Proteccion Familiar/Estrategia/Estrategia 2026/3.Estrategia Comercial 2026/Dash board/Archivos 18032026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos de Mes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D559B825-2D31-4392-A448-10C4A0CB90AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{D559B825-2D31-4392-A448-10C4A0CB90AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAC15A40-8EFE-4E7F-A118-91CF8DBEA79E}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{40BDA7B1-706D-4201-BBD8-6F9F96398CA1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{40BDA7B1-706D-4201-BBD8-6F9F96398CA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Comisiones Asesores" sheetId="1" r:id="rId1"/>
@@ -80,9 +80,6 @@
     <t>13 a 36</t>
   </si>
   <si>
-    <t>37 a 60</t>
-  </si>
-  <si>
     <t>60 a mas</t>
   </si>
   <si>
@@ -111,6 +108,9 @@
   </si>
   <si>
     <t>Pie</t>
+  </si>
+  <si>
+    <t>37 a 59</t>
   </si>
 </sst>
 </file>
@@ -694,15 +694,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BAC097C-142B-4AEA-A0F1-6992D46CDB83}">
   <dimension ref="A1:E23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.86328125" customWidth="1"/>
-    <col min="5" max="5" width="21.3984375" customWidth="1"/>
+    <col min="4" max="4" width="17.88671875" customWidth="1"/>
+    <col min="5" max="5" width="21.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -712,7 +712,7 @@
       </c>
       <c r="E1" s="8"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -726,7 +726,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -740,7 +740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -754,7 +754,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -768,53 +768,53 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B6" s="3">
         <v>0.08</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E6" s="3">
         <v>0.01</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" s="3">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E7" s="3">
         <v>0.01</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>5</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>10</v>
@@ -823,9 +823,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15" s="4">
         <v>0.125</v>
@@ -837,7 +837,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -849,7 +849,7 @@
       </c>
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>7</v>
       </c>
@@ -861,7 +861,7 @@
       </c>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -873,9 +873,9 @@
       </c>
       <c r="D18" s="4"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" s="4">
         <v>0.125</v>
@@ -883,9 +883,9 @@
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" s="4">
         <v>0.125</v>
@@ -893,9 +893,9 @@
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" s="4">
         <v>0.125</v>
@@ -903,9 +903,9 @@
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22" s="4">
         <v>0.125</v>
@@ -913,9 +913,9 @@
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B23" s="7">
         <f>SUM(B14:B22)</f>

</xml_diff>